<commit_message>
feat: rewrite RtgsneftEntry (TRANSACTIONMST) with real CBS field IDs from live DOM — replace invented RTGS/NEFT files with unified RtgsNeftEntryPage, Builder, Repository, Validator and all 5 specs
</commit_message>
<xml_diff>
--- a/src/modules/Transaction/RtgsAndNeft/RtgsneftEntry/data/RtgsneftEntry.xlsx
+++ b/src/modules/Transaction/RtgsAndNeft/RtgsneftEntry/data/RtgsneftEntry.xlsx
@@ -5,91 +5,249 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Create" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Update" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Authorize" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Negative" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Database" state="visible" r:id="rId8"/>
+    <sheet sheetId="2" name="Auth" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Update" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Database" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
-  <si>
-    <t>debitAccountNumber</t>
-  </si>
-  <si>
-    <t>beneficiaryName</t>
-  </si>
-  <si>
-    <t>beneficiaryAccountNumber</t>
-  </si>
-  <si>
-    <t>beneficiaryIFSC</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="78">
+  <si>
+    <t>msgTrfType</t>
+  </si>
+  <si>
+    <t>msgSType</t>
+  </si>
+  <si>
+    <t>msgDate</t>
+  </si>
+  <si>
+    <t>rtgsNeftAcctId</t>
+  </si>
+  <si>
+    <t>tBatchCd</t>
+  </si>
+  <si>
+    <t>ordIFSCCd</t>
+  </si>
+  <si>
+    <t>orgBrCode</t>
+  </si>
+  <si>
+    <t>ordAcctId</t>
+  </si>
+  <si>
+    <t>ordDesc1</t>
+  </si>
+  <si>
+    <t>ordDesc2</t>
+  </si>
+  <si>
+    <t>ordDesc3</t>
+  </si>
+  <si>
+    <t>mobileEmail</t>
+  </si>
+  <si>
+    <t>mobileNo</t>
+  </si>
+  <si>
+    <t>insType</t>
+  </si>
+  <si>
+    <t>chequeNo</t>
+  </si>
+  <si>
+    <t>instrDate</t>
+  </si>
+  <si>
+    <t>insDate</t>
+  </si>
+  <si>
+    <t>valueAmt_txt</t>
+  </si>
+  <si>
+    <t>cusLeiNo</t>
+  </si>
+  <si>
+    <t>benLeiNo</t>
+  </si>
+  <si>
+    <t>organisationCode</t>
+  </si>
+  <si>
+    <t>dtlsOfChrgs</t>
+  </si>
+  <si>
+    <t>msgPriority</t>
+  </si>
+  <si>
+    <t>benIFSCCd</t>
+  </si>
+  <si>
+    <t>benDesc1</t>
+  </si>
+  <si>
+    <t>benDesc2</t>
+  </si>
+  <si>
+    <t>benDesc3</t>
+  </si>
+  <si>
+    <t>fldNo</t>
+  </si>
+  <si>
+    <t>fld1</t>
+  </si>
+  <si>
+    <t>1=RTGS 2=NEFT</t>
+  </si>
+  <si>
+    <t>N06=NEFT OUT R41=CUST PMT</t>
+  </si>
+  <si>
+    <t>dd-mm-yyyy</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>e.g. KKBK0000261</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Automation Ordering Customer</t>
+  </si>
+  <si>
+    <t>1=MOBILE 2=EMAIL</t>
+  </si>
+  <si>
+    <t>10 digits</t>
+  </si>
+  <si>
+    <t>99=VOUCHER</t>
   </si>
   <si>
     <t>amount</t>
   </si>
   <si>
-    <t>remarks</t>
-  </si>
-  <si>
-    <t>ACC001234567</t>
+    <t>e.g. SBIN0001234</t>
+  </si>
+  <si>
+    <t>14 digit acct</t>
+  </si>
+  <si>
+    <t>Beneficiary Name</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>7023=PAYMENT DETAILS</t>
+  </si>
+  <si>
+    <t>Payment remarks</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>N06</t>
+  </si>
+  <si>
+    <t>KKBK0000261</t>
+  </si>
+  <si>
+    <t>Test Ordering Customer</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>SBIN0001234</t>
+  </si>
+  <si>
+    <t>12345678901234</t>
   </si>
   <si>
     <t>Test Beneficiary</t>
   </si>
   <si>
-    <t>98765432109876</t>
-  </si>
-  <si>
-    <t>HDFC0001234</t>
-  </si>
-  <si>
-    <t>500000</t>
-  </si>
-  <si>
-    <t>Automation Test</t>
-  </si>
-  <si>
-    <t>transactionRef</t>
-  </si>
-  <si>
-    <t>TXN001</t>
-  </si>
-  <si>
-    <t>Updated remarks</t>
-  </si>
-  <si>
-    <t>expectedStatus</t>
-  </si>
-  <si>
-    <t>AUTHORIZED</t>
-  </si>
-  <si>
-    <t>scenario</t>
-  </si>
-  <si>
-    <t>expectedError</t>
-  </si>
-  <si>
-    <t>Below Minimum</t>
-  </si>
-  <si>
-    <t>100000</t>
-  </si>
-  <si>
-    <t>Invalid IFSC</t>
-  </si>
-  <si>
-    <t>INVALID</t>
-  </si>
-  <si>
-    <t>expectedAmount</t>
-  </si>
-  <si>
-    <t>PROCESSED</t>
+    <t>Test Address</t>
+  </si>
+  <si>
+    <t>7023</t>
+  </si>
+  <si>
+    <t>Automation NEFT payment</t>
+  </si>
+  <si>
+    <t>R41</t>
+  </si>
+  <si>
+    <t>200000</t>
+  </si>
+  <si>
+    <t>Automation RTGS payment</t>
+  </si>
+  <si>
+    <t>searchKey</t>
+  </si>
+  <si>
+    <t>tab</t>
+  </si>
+  <si>
+    <t>notes: searchKey = rtgsNeftAcctId or benDesc1 from create</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>notes: searchKey from create result</t>
+  </si>
+  <si>
+    <t>updated amount</t>
+  </si>
+  <si>
+    <t>updated name</t>
+  </si>
+  <si>
+    <t>updated remarks</t>
+  </si>
+  <si>
+    <t>15000</t>
+  </si>
+  <si>
+    <t>Updated Beneficiary</t>
+  </si>
+  <si>
+    <t>Updated payment remarks</t>
+  </si>
+  <si>
+    <t>setNo</t>
+  </si>
+  <si>
+    <t>scrollNo</t>
+  </si>
+  <si>
+    <t>notes: setNo or scrollNo captured after create</t>
   </si>
 </sst>
 </file>
@@ -466,10 +624,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,25 +646,341 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>34</v>
+      </c>
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T2" t="s">
+        <v>32</v>
+      </c>
+      <c r="U2" t="s">
+        <v>32</v>
+      </c>
+      <c r="V2" t="s">
+        <v>32</v>
+      </c>
+      <c r="W2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R3" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" t="s">
+        <v>32</v>
+      </c>
+      <c r="T3" t="s">
+        <v>32</v>
+      </c>
+      <c r="U3" t="s">
+        <v>32</v>
+      </c>
+      <c r="V3" t="s">
+        <v>32</v>
+      </c>
+      <c r="W3" t="s">
+        <v>32</v>
+      </c>
+      <c r="X3" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" t="s">
+        <v>32</v>
+      </c>
+      <c r="P4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R4" t="s">
+        <v>62</v>
+      </c>
+      <c r="S4" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" t="s">
+        <v>32</v>
+      </c>
+      <c r="U4" t="s">
+        <v>32</v>
+      </c>
+      <c r="V4" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" t="s">
+        <v>32</v>
+      </c>
+      <c r="X4" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -517,23 +991,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -544,23 +1026,58 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -571,82 +1088,31 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>